<commit_message>
Update client outreach templates with live Vercel domain
</commit_message>
<xml_diff>
--- a/devduo_global_leads_50.xlsx
+++ b/devduo_global_leads_50.xlsx
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="G2" s="7">
-        <f>HYPERLINK("https://wa.me/971543470278?text=Hi%20A-One%20Web%20Design%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971543470278?text=Hi%20A-One%20Web%20Design%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -614,7 +614,7 @@
       <c r="I2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi A-One Web Design team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="G3" s="7">
-        <f>HYPERLINK("https://wa.me/971506063996?text=Hi%20Woxier%20Digital%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971506063996?text=Hi%20Woxier%20Digital%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -674,7 +674,7 @@
       <c r="I3" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Woxier Digital team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="G4" s="7">
-        <f>HYPERLINK("https://wa.me/971544012919?text=Hi%20Creative971%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971544012919?text=Hi%20Creative971%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -734,7 +734,7 @@
       <c r="I4" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Creative971 team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="G5" s="7">
-        <f>HYPERLINK("https://wa.me/971555515475?text=Hi%20Dubai%20Web%20Design%20%28DWD%29%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971555515475?text=Hi%20Dubai%20Web%20Design%20%28DWD%29%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -794,7 +794,7 @@
       <c r="I5" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Dubai Web Design (DWD) team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="G6" s="7">
-        <f>HYPERLINK("https://wa.me/971551353016?text=Hi%20Digiant%20Media%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971551353016?text=Hi%20Digiant%20Media%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -854,7 +854,7 @@
       <c r="I6" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Digiant Media team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -903,7 +903,7 @@
         </is>
       </c>
       <c r="G7" s="7">
-        <f>HYPERLINK("https://wa.me/971508371091?text=Hi%20Digital%20Advengers%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971508371091?text=Hi%20Digital%20Advengers%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -914,7 +914,7 @@
       <c r="I7" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Digital Advengers team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="G8" s="7">
-        <f>HYPERLINK("https://wa.me/971568491313?text=Hi%20Easywebplans%20IT%20LLC%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971568491313?text=Hi%20Easywebplans%20IT%20LLC%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -974,7 +974,7 @@
       <c r="I8" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Easywebplans IT LLC team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="G9" s="7">
-        <f>HYPERLINK("https://wa.me/971545430169?text=Hi%20Nile%20Web%20Agency%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971545430169?text=Hi%20Nile%20Web%20Agency%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1034,7 +1034,7 @@
       <c r="I9" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Nile Web Agency team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="G10" s="7">
-        <f>HYPERLINK("https://wa.me/971503047470?text=Hi%20Leads%20Dubai%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971503047470?text=Hi%20Leads%20Dubai%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1094,7 +1094,7 @@
       <c r="I10" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Leads Dubai team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="G11" s="7">
-        <f>HYPERLINK("https://wa.me/971507867884?text=Hi%20Digital%20Media%20Sapiens%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971507867884?text=Hi%20Digital%20Media%20Sapiens%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1154,7 +1154,7 @@
       <c r="I11" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Digital Media Sapiens team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="G12" s="7">
-        <f>HYPERLINK("https://wa.me/971544875436?text=Hi%20A2Z%20Webinfotech%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971544875436?text=Hi%20A2Z%20Webinfotech%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1214,7 +1214,7 @@
       <c r="I12" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi A2Z Webinfotech team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1263,7 +1263,7 @@
         </is>
       </c>
       <c r="G13" s="7">
-        <f>HYPERLINK("https://wa.me/971555212254?text=Hi%20Lead%20Smart%20Web%20Solutions%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971555212254?text=Hi%20Lead%20Smart%20Web%20Solutions%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1274,7 +1274,7 @@
       <c r="I13" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Lead Smart Web Solutions team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="G14" s="7">
-        <f>HYPERLINK("https://wa.me/971505705820?text=Hi%20Aquaholic%20Solutions%20%28AQ%29%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971505705820?text=Hi%20Aquaholic%20Solutions%20%28AQ%29%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1334,7 +1334,7 @@
       <c r="I14" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Aquaholic Solutions (AQ) team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="G15" s="7">
-        <f>HYPERLINK("https://wa.me/971508482289?text=Hi%20Abu%20Dhabi%20Digital%20Tech%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971508482289?text=Hi%20Abu%20Dhabi%20Digital%20Tech%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1394,7 +1394,7 @@
       <c r="I15" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Abu Dhabi Digital Tech team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1443,7 +1443,7 @@
         </is>
       </c>
       <c r="G16" s="7">
-        <f>HYPERLINK("https://wa.me/971542858955?text=Hi%20General%20Tech%20%26%20Design%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/971542858955?text=Hi%20General%20Tech%20%26%20Design%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1454,7 +1454,7 @@
       <c r="I16" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi General Tech &amp; Design team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1503,7 +1503,7 @@
         </is>
       </c>
       <c r="G17" s="7">
-        <f>HYPERLINK("https://wa.me/966539969700?text=Hi%20Digital%20Growth%20Solutions%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/966539969700?text=Hi%20Digital%20Growth%20Solutions%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1514,7 +1514,7 @@
       <c r="I17" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Digital Growth Solutions team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="G18" s="7">
-        <f>HYPERLINK("https://wa.me/966564229190?text=Hi%20Local%20City%20Solutions%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/966564229190?text=Hi%20Local%20City%20Solutions%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1574,7 +1574,7 @@
       <c r="I18" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Local City Solutions team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1623,7 +1623,7 @@
         </is>
       </c>
       <c r="G19" s="7">
-        <f>HYPERLINK("https://wa.me/966536069636?text=Hi%20Crayo%20Tech%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/966536069636?text=Hi%20Crayo%20Tech%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1634,7 +1634,7 @@
       <c r="I19" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Crayo Tech team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1683,7 +1683,7 @@
         </is>
       </c>
       <c r="G20" s="7">
-        <f>HYPERLINK("https://wa.me/966577975969?text=Hi%20Web%20Design%20KSA%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/966577975969?text=Hi%20Web%20Design%20KSA%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1694,7 +1694,7 @@
       <c r="I20" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Web Design KSA team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1743,7 +1743,7 @@
         </is>
       </c>
       <c r="G21" s="7">
-        <f>HYPERLINK("https://wa.me/966508376256?text=Hi%20Wisoft%20Solutions%20KSA%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/966508376256?text=Hi%20Wisoft%20Solutions%20KSA%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1754,7 +1754,7 @@
       <c r="I21" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Wisoft Solutions KSA team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1803,7 +1803,7 @@
         </is>
       </c>
       <c r="G22" s="7">
-        <f>HYPERLINK("https://wa.me/966551238910?text=Hi%20Safha%20Tech%20Studio%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/966551238910?text=Hi%20Safha%20Tech%20Studio%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1814,7 +1814,7 @@
       <c r="I22" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Safha Tech Studio team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1863,7 +1863,7 @@
         </is>
       </c>
       <c r="G23" s="7">
-        <f>HYPERLINK("https://wa.me/966541298741?text=Hi%20Bytes%20Future%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/966541298741?text=Hi%20Bytes%20Future%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1874,7 +1874,7 @@
       <c r="I23" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Bytes Future team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1923,7 +1923,7 @@
         </is>
       </c>
       <c r="G24" s="7">
-        <f>HYPERLINK("https://wa.me/966509871234?text=Hi%20Standard%20Touch%20KSA%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/966509871234?text=Hi%20Standard%20Touch%20KSA%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -1934,7 +1934,7 @@
       <c r="I24" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Standard Touch KSA team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -1983,7 +1983,7 @@
         </is>
       </c>
       <c r="G25" s="7">
-        <f>HYPERLINK("https://wa.me/966538901245?text=Hi%20Al-Bayan%20Digital%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/966538901245?text=Hi%20Al-Bayan%20Digital%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1994,7 +1994,7 @@
       <c r="I25" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Al-Bayan Digital team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="G26" s="7">
-        <f>HYPERLINK("https://wa.me/966567891230?text=Hi%20Riyadh%20Web%20Creators%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/966567891230?text=Hi%20Riyadh%20Web%20Creators%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -2054,7 +2054,7 @@
       <c r="I26" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Riyadh Web Creators team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="G27" s="7">
-        <f>HYPERLINK("https://wa.me/97431453222?text=Hi%20Artisans%20Digital%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/97431453222?text=Hi%20Artisans%20Digital%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -2114,7 +2114,7 @@
       <c r="I27" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Artisans Digital team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -2163,7 +2163,7 @@
         </is>
       </c>
       <c r="G28" s="7">
-        <f>HYPERLINK("https://wa.me/97431096699?text=Hi%20Creative%20Web%20Design%20Qatar%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/97431096699?text=Hi%20Creative%20Web%20Design%20Qatar%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -2174,7 +2174,7 @@
       <c r="I28" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Creative Web Design Qatar team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -2223,7 +2223,7 @@
         </is>
       </c>
       <c r="G29" s="7">
-        <f>HYPERLINK("https://wa.me/97433176825?text=Hi%20PTC%20Media%20Qatar%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/97433176825?text=Hi%20PTC%20Media%20Qatar%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -2234,7 +2234,7 @@
       <c r="I29" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi PTC Media Qatar team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -2283,7 +2283,7 @@
         </is>
       </c>
       <c r="G30" s="7">
-        <f>HYPERLINK("https://wa.me/97472045132?text=Hi%20Web%20Design%20Agency%20Doha%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/97472045132?text=Hi%20Web%20Design%20Agency%20Doha%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -2294,7 +2294,7 @@
       <c r="I30" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Web Design Agency Doha team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -2343,7 +2343,7 @@
         </is>
       </c>
       <c r="G31" s="7">
-        <f>HYPERLINK("https://wa.me/96565534477?text=Hi%20Kuwait%20Web%20Design%20%28KWD%29%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/96565534477?text=Hi%20Kuwait%20Web%20Design%20%28KWD%29%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H31" s="4" t="inlineStr">
@@ -2354,7 +2354,7 @@
       <c r="I31" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Kuwait Web Design (KWD) team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -2403,7 +2403,7 @@
         </is>
       </c>
       <c r="G32" s="7">
-        <f>HYPERLINK("https://wa.me/96522923456?text=Hi%20MAK%20United%20Tech%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/96522923456?text=Hi%20MAK%20United%20Tech%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2414,7 +2414,7 @@
       <c r="I32" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi MAK United Tech team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="G33" s="7">
-        <f>HYPERLINK("https://wa.me/97335460525?text=Hi%20Friend%20Tech%20IT%20Solutions%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/97335460525?text=Hi%20Friend%20Tech%20IT%20Solutions%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -2474,7 +2474,7 @@
       <c r="I33" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Friend Tech IT Solutions team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="G34" s="7">
-        <f>HYPERLINK("https://wa.me/97339246555?text=Hi%20Info%20Bahrain%20Web%20Design%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/97339246555?text=Hi%20Info%20Bahrain%20Web%20Design%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -2534,7 +2534,7 @@
       <c r="I34" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Info Bahrain Web Design team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -2583,7 +2583,7 @@
         </is>
       </c>
       <c r="G35" s="7">
-        <f>HYPERLINK("https://wa.me/97317712313?text=Hi%20Breakthrough%20Digital%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
+        <f>HYPERLINK("https://wa.me/97317712313?text=Hi%20Breakthrough%20Digital%20team%21%20%F0%9F%91%8B%0A%0AI%27m%20Imran%2C%20co-founder%20at%20DEVDUO%20Studio%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Frontend%20Engineer%29.%0A%0AWe%20partner%20with%20digital%20and%20creative%20agencies%20across%20the%20Gulf%20and%20globally%20as%20a%20dedicated%20white-label%20engineering%20arm.%20When%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20systems%2C%20we%20build%20them%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20engineers%20%28clean%20architecture%2C%2014ms%20API%20latency%29%0A%E2%80%A2%20Fast%20turnarounds%20%28MVPs%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Complete%20privacy%20%26%20white-label%20delivery%0A%0AAre%20you%20open%20to%20having%20a%20reliable%20technical%20partner%20for%20your%20upcoming%20client%20projects%3F%0A%0ABest%20regards%2C%0AImran%20%26%20Mubin%20%7C%20DEVDUO%0ATelegram%3A%20%40rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "💬 Открыть WhatsApp")</f>
         <v/>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -2594,7 +2594,7 @@
       <c r="I35" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hi Breakthrough Digital team! 👋
-I'm Imran, co-founder at DEVDUO Studio (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
+I'm Imran, co-founder at DEVDUO Studio (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Frontend Engineer).
 We partner with digital and creative agencies across the Gulf and globally as a dedicated white-label engineering arm. When you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI systems, we build them under your brand:
 • 100% Senior engineers (clean architecture, 14ms API latency)
 • Fast turnarounds (MVPs in 2–4 weeks, fixed sprints from $490)
@@ -2643,7 +2643,7 @@
         </is>
       </c>
       <c r="G36" s="7">
-        <f>HYPERLINK("mailto:info@klashtech.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Klashtech%20Digital%20Agency&amp;body=Hi%20Klashtech%20Digital%20Agency%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:info@klashtech.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Klashtech%20Digital%20Agency&amp;body=Hi%20Klashtech%20Digital%20Agency%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -2655,7 +2655,7 @@
         <is>
           <t xml:space="preserve">Hi Klashtech Digital Agency team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -2664,7 +2664,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -2706,7 +2706,7 @@
         </is>
       </c>
       <c r="G37" s="7">
-        <f>HYPERLINK("mailto:hello@hmgcreative.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20HMG%20Creative&amp;body=Hi%20HMG%20Creative%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:hello@hmgcreative.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20HMG%20Creative&amp;body=Hi%20HMG%20Creative%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -2718,7 +2718,7 @@
         <is>
           <t xml:space="preserve">Hi HMG Creative team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -2727,7 +2727,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="G38" s="7">
-        <f>HYPERLINK("mailto:contact@devoxsoftware.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Devox%20Software&amp;body=Hi%20Devox%20Software%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:contact@devoxsoftware.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Devox%20Software&amp;body=Hi%20Devox%20Software%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -2781,7 +2781,7 @@
         <is>
           <t xml:space="preserve">Hi Devox Software team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -2790,7 +2790,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -2832,7 +2832,7 @@
         </is>
       </c>
       <c r="G39" s="7">
-        <f>HYPERLINK("mailto:hello@lovelygrit.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Lovely%20Grit&amp;body=Hi%20Lovely%20Grit%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:hello@lovelygrit.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Lovely%20Grit&amp;body=Hi%20Lovely%20Grit%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -2844,7 +2844,7 @@
         <is>
           <t xml:space="preserve">Hi Lovely Grit team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -2853,7 +2853,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -2895,7 +2895,7 @@
         </is>
       </c>
       <c r="G40" s="7">
-        <f>HYPERLINK("mailto:info@WDCagency.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20WDC%20Agency&amp;body=Hi%20WDC%20Agency%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:info@WDCagency.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20WDC%20Agency&amp;body=Hi%20WDC%20Agency%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -2907,7 +2907,7 @@
         <is>
           <t xml:space="preserve">Hi WDC Agency team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -2916,7 +2916,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -2958,7 +2958,7 @@
         </is>
       </c>
       <c r="G41" s="7">
-        <f>HYPERLINK("mailto:hello@dd.nyc?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20DD.NYC&amp;body=Hi%20DD.NYC%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:hello@dd.nyc?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20DD.NYC&amp;body=Hi%20DD.NYC%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -2970,7 +2970,7 @@
         <is>
           <t xml:space="preserve">Hi DD.NYC team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -2979,7 +2979,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3021,7 +3021,7 @@
         </is>
       </c>
       <c r="G42" s="7">
-        <f>HYPERLINK("mailto:hello@bowenmedia.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Bowen%20Media&amp;body=Hi%20Bowen%20Media%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:hello@bowenmedia.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Bowen%20Media&amp;body=Hi%20Bowen%20Media%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -3033,7 +3033,7 @@
         <is>
           <t xml:space="preserve">Hi Bowen Media team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3042,7 +3042,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3084,7 +3084,7 @@
         </is>
       </c>
       <c r="G43" s="7">
-        <f>HYPERLINK("mailto:info@netlynxinc.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Netlynx%20Inc&amp;body=Hi%20Netlynx%20Inc%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:info@netlynxinc.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Netlynx%20Inc&amp;body=Hi%20Netlynx%20Inc%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -3096,7 +3096,7 @@
         <is>
           <t xml:space="preserve">Hi Netlynx Inc team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3105,7 +3105,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3147,7 +3147,7 @@
         </is>
       </c>
       <c r="G44" s="7">
-        <f>HYPERLINK("mailto:info@fuze360.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20FUZE%20Agency&amp;body=Hi%20FUZE%20Agency%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:info@fuze360.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20FUZE%20Agency&amp;body=Hi%20FUZE%20Agency%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -3159,7 +3159,7 @@
         <is>
           <t xml:space="preserve">Hi FUZE Agency team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3168,7 +3168,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3210,7 +3210,7 @@
         </is>
       </c>
       <c r="G45" s="7">
-        <f>HYPERLINK("mailto:info@gallagherwebsitedesign.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Gallagher%20Website%20Design&amp;body=Hi%20Gallagher%20Website%20Design%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:info@gallagherwebsitedesign.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Gallagher%20Website%20Design&amp;body=Hi%20Gallagher%20Website%20Design%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H45" s="4" t="inlineStr">
@@ -3222,7 +3222,7 @@
         <is>
           <t xml:space="preserve">Hi Gallagher Website Design team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3231,7 +3231,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="G46" s="7">
-        <f>HYPERLINK("mailto:hello@rocketair.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20RocketAir%20Design&amp;body=Hi%20RocketAir%20Design%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:hello@rocketair.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20RocketAir%20Design&amp;body=Hi%20RocketAir%20Design%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H46" s="4" t="inlineStr">
@@ -3285,7 +3285,7 @@
         <is>
           <t xml:space="preserve">Hi RocketAir Design team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3294,7 +3294,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3336,7 +3336,7 @@
         </is>
       </c>
       <c r="G47" s="7">
-        <f>HYPERLINK("mailto:hello@clay.global?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Clay%20Global&amp;body=Hi%20Clay%20Global%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:hello@clay.global?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Clay%20Global&amp;body=Hi%20Clay%20Global%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H47" s="4" t="inlineStr">
@@ -3348,7 +3348,7 @@
         <is>
           <t xml:space="preserve">Hi Clay Global team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3357,7 +3357,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3399,7 +3399,7 @@
         </is>
       </c>
       <c r="G48" s="7">
-        <f>HYPERLINK("mailto:hello@designboutiqueuk.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Design%20Boutique%20UK&amp;body=Hi%20Design%20Boutique%20UK%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:hello@designboutiqueuk.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Design%20Boutique%20UK&amp;body=Hi%20Design%20Boutique%20UK%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H48" s="4" t="inlineStr">
@@ -3411,7 +3411,7 @@
         <is>
           <t xml:space="preserve">Hi Design Boutique UK team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3420,7 +3420,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3462,7 +3462,7 @@
         </is>
       </c>
       <c r="G49" s="7">
-        <f>HYPERLINK("mailto:hello@digitali.co.uk?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Digitali%20Studio&amp;body=Hi%20Digitali%20Studio%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:hello@digitali.co.uk?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Digitali%20Studio&amp;body=Hi%20Digitali%20Studio%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H49" s="4" t="inlineStr">
@@ -3474,7 +3474,7 @@
         <is>
           <t xml:space="preserve">Hi Digitali Studio team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3483,7 +3483,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="G50" s="7">
-        <f>HYPERLINK("mailto:info@fellowstudio.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Fellow%20Studio&amp;body=Hi%20Fellow%20Studio%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:info@fellowstudio.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Fellow%20Studio&amp;body=Hi%20Fellow%20Studio%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H50" s="4" t="inlineStr">
@@ -3537,7 +3537,7 @@
         <is>
           <t xml:space="preserve">Hi Fellow Studio team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3546,7 +3546,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3588,7 +3588,7 @@
         </is>
       </c>
       <c r="G51" s="7">
-        <f>HYPERLINK("mailto:hello@minttwist.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20MintTwist&amp;body=Hi%20MintTwist%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:hello@minttwist.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20MintTwist&amp;body=Hi%20MintTwist%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H51" s="4" t="inlineStr">
@@ -3600,7 +3600,7 @@
         <is>
           <t xml:space="preserve">Hi MintTwist team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3609,7 +3609,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3651,7 +3651,7 @@
         </is>
       </c>
       <c r="G52" s="7">
-        <f>HYPERLINK("mailto:info@webheads.co.uk?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Webheads&amp;body=Hi%20Webheads%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:info@webheads.co.uk?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Webheads&amp;body=Hi%20Webheads%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H52" s="4" t="inlineStr">
@@ -3663,7 +3663,7 @@
         <is>
           <t xml:space="preserve">Hi Webheads team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3672,7 +3672,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3714,7 +3714,7 @@
         </is>
       </c>
       <c r="G53" s="7">
-        <f>HYPERLINK("mailto:enquiries@webprocreative.co.uk?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20WEBPRO%20Creative&amp;body=Hi%20WEBPRO%20Creative%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:enquiries@webprocreative.co.uk?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20WEBPRO%20Creative&amp;body=Hi%20WEBPRO%20Creative%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H53" s="4" t="inlineStr">
@@ -3726,7 +3726,7 @@
         <is>
           <t xml:space="preserve">Hi WEBPRO Creative team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3735,7 +3735,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3777,7 +3777,7 @@
         </is>
       </c>
       <c r="G54" s="7">
-        <f>HYPERLINK("mailto:hello@buildinamsterdam.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Build%20in%20Amsterdam&amp;body=Hi%20Build%20in%20Amsterdam%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:hello@buildinamsterdam.com?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Build%20in%20Amsterdam&amp;body=Hi%20Build%20in%20Amsterdam%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H54" s="4" t="inlineStr">
@@ -3789,7 +3789,7 @@
         <is>
           <t xml:space="preserve">Hi Build in Amsterdam team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3798,7 +3798,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>
@@ -3840,7 +3840,7 @@
         </is>
       </c>
       <c r="G55" s="7">
-        <f>HYPERLINK("mailto:hello@brandium.nl?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Brandium%20Agency&amp;body=Hi%20Brandium%20Agency%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//imron-backend-frotend.github.io/devduo-agency/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//imron-backend-frotend.github.io/devduo-agency/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
+        <f>HYPERLINK("mailto:hello@brandium.nl?subject=Dev%20partnership%20/%20White-label%20engineering%20for%20Brandium%20Agency&amp;body=Hi%20Brandium%20Agency%20team%2C%0A%0AI%E2%80%99ve%20been%20following%20your%20work%20and%20really%20admire%20the%20digital%20experiences%20and%20products%20you%20deliver.%0A%0AI%E2%80%99m%20Imran%2C%20co-founder%20at%20DEVDUO%20%28https%3A//devduo-studio.vercel.app/en/%29.%20We%20are%20an%20engineering%20studio%20of%20two%20senior%20developers%20%28Lead%20Backend%20Architect%20%2B%20Senior%20Product%20Engineer%29.%0A%0AWe%20partner%20with%20creative%20and%20digital%20agencies%20in%20the%20US%2C%20UK%2C%20and%20Europe%20as%20a%20dedicated%20white-label%20engineering%20arm.%20Whenever%20you%20need%20custom%20web%20platforms%2C%20complex%20backends%20%28FastAPI/Python/Node%29%2C%20or%20mobile/AI%20integrations%2C%20we%20build%20the%20technical%20side%20under%20your%20brand%3A%0A%0A%E2%80%A2%20100%25%20Senior%20Engineers%20%28zero%20junior%20handoffs%20or%20PM%20bloat%29%0A%E2%80%A2%20High%20velocity%20%28MVPs%20shipped%20in%202%E2%80%934%20weeks%2C%20fixed%20sprints%20from%20%24490%29%0A%E2%80%A2%20Production-grade%20stack%3A%20React%2019%2C%20Next.js%2C%20Python%2C%20PostgreSQL%2C%20Docker%2C%20AI/LLMs%0A%0AWould%20you%20be%20open%20to%20a%20quick%2010-minute%20chat%20or%20async%20message%20exchange%20to%20see%20if%20we%20could%20support%20your%20upcoming%20project%20pipeline%3F%0A%0ABest%20regards%2C%0A%0AImran%20%26%20Mubin%0AFounders%20%26%20Senior%20Engineers%20%7C%20DEVDUO%20Studio%0APortfolio%3A%20https%3A//devduo-studio.vercel.app/en/%0ATelegram%3A%20https%3A//t.me/rolldurov%0AEmail%3A%20devduo.engineering%40gmail.com%0A", "✉️ Отправить Email")</f>
         <v/>
       </c>
       <c r="H55" s="4" t="inlineStr">
@@ -3852,7 +3852,7 @@
         <is>
           <t xml:space="preserve">Hi Brandium Agency team,
 I’ve been following your work and really admire the digital experiences and products you deliver.
-I’m Imran, co-founder at DEVDUO (https://imron-backend-frotend.github.io/devduo-agency/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
+I’m Imran, co-founder at DEVDUO (https://devduo-studio.vercel.app/en/). We are an engineering studio of two senior developers (Lead Backend Architect + Senior Product Engineer).
 We partner with creative and digital agencies in the US, UK, and Europe as a dedicated white-label engineering arm. Whenever you need custom web platforms, complex backends (FastAPI/Python/Node), or mobile/AI integrations, we build the technical side under your brand:
 • 100% Senior Engineers (zero junior handoffs or PM bloat)
 • High velocity (MVPs shipped in 2–4 weeks, fixed sprints from $490)
@@ -3861,7 +3861,7 @@
 Best regards,
 Imran &amp; Mubin
 Founders &amp; Senior Engineers | DEVDUO Studio
-Portfolio: https://imron-backend-frotend.github.io/devduo-agency/en/
+Portfolio: https://devduo-studio.vercel.app/en/
 Telegram: https://t.me/rolldurov
 Email: devduo.engineering@gmail.com
 </t>

</xml_diff>